<commit_message>
Reports save bug fix
</commit_message>
<xml_diff>
--- a/CafeApp/Resources/AdminReport.xlsx
+++ b/CafeApp/Resources/AdminReport.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikit\Downloads\Telegram Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RiderProjects\CafeApp\CafeApp\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8AA5863-A907-4075-90A8-EB886EFFE951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D04AAED-A662-4771-8581-422311EE776B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{7527AC48-548A-4BA7-8058-2E3AE9E8A996}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Заказ</t>
   </si>
@@ -44,6 +44,9 @@
   </si>
   <si>
     <t>Выполнен в</t>
+  </si>
+  <si>
+    <t>Метод оплаты</t>
   </si>
 </sst>
 </file>
@@ -80,15 +83,9 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -98,9 +95,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -437,16 +437,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AA25714-41BC-4788-8AEF-D819481E67F9}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="17.6640625" customWidth="1"/>
     <col min="4" max="4" width="26.5546875" customWidth="1"/>
     <col min="5" max="5" width="17.6640625" customWidth="1"/>
-    <col min="7" max="8" width="17.6640625" customWidth="1"/>
+    <col min="7" max="9" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -470,6 +470,9 @@
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>